<commit_message>
Update Excel source and regenerate migration scripts
- Fetch corrected 데이터원본_2602.xlsx from main (2025-05, 06 zeros fixed)
- Regenerate paste-in-console.js and migration-payload.json

https://claude.ai/code/session_01PaVG4UWgZ541676uvc2w4y
</commit_message>
<xml_diff>
--- a/데이터원본_2602.xlsx
+++ b/데이터원본_2602.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\내 드라이브\02_AREA\04_재무\04_연금전략 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB35927F-ED50-426C-8E7D-AB2B84FCE6BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{577F5B33-3C1A-416F-9B5E-1D6658105B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34070" yWindow="-12580" windowWidth="19200" windowHeight="11180" activeTab="2" xr2:uid="{182F7363-D65B-489E-BF18-685EC1FD72DA}"/>
+    <workbookView xWindow="-38350" yWindow="-16110" windowWidth="38620" windowHeight="15500" xr2:uid="{182F7363-D65B-489E-BF18-685EC1FD72DA}"/>
   </bookViews>
   <sheets>
     <sheet name="평가금액" sheetId="1" r:id="rId1"/>
@@ -10773,8 +10773,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78ADBEF8-D366-4094-B208-FBD4D5A79444}">
-  <dimension ref="A1:J104"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="10.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.08203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.4140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.75" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.75" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.08203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B1" t="s">
@@ -13333,7 +13345,7 @@
         <v>17413895</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A81" s="1">
         <v>45382</v>
       </c>
@@ -13365,7 +13377,7 @@
         <v>17555497</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A82" s="1">
         <v>45412</v>
       </c>
@@ -13397,7 +13409,7 @@
         <v>17326323</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A83" s="1">
         <v>45443</v>
       </c>
@@ -13429,7 +13441,7 @@
         <v>17432553</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A84" s="1">
         <v>45473</v>
       </c>
@@ -13461,7 +13473,7 @@
         <v>17415122</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A85" s="1">
         <v>45504</v>
       </c>
@@ -13493,7 +13505,7 @@
         <v>13084610</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A86" s="1">
         <v>45535</v>
       </c>
@@ -13525,7 +13537,7 @@
         <v>8220953</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A87" s="1">
         <v>45565</v>
       </c>
@@ -13557,7 +13569,7 @@
         <v>4396464</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A88" s="1">
         <v>45596</v>
       </c>
@@ -13589,7 +13601,7 @@
         <v>4032135</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A89" s="1">
         <v>45626</v>
       </c>
@@ -13621,7 +13633,7 @@
         <v>1650487</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A90" s="1">
         <v>45657</v>
       </c>
@@ -13653,7 +13665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A91" s="1">
         <v>45688</v>
       </c>
@@ -13685,7 +13697,7 @@
         <v>1750</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A92" s="1">
         <v>45716</v>
       </c>
@@ -13717,7 +13729,7 @@
         <v>1750</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A93" s="1">
         <v>45747</v>
       </c>
@@ -13749,7 +13761,7 @@
         <v>1750</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A94" s="1">
         <v>45777</v>
       </c>
@@ -13781,69 +13793,71 @@
         <v>1750</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A95" s="1">
         <v>45808</v>
       </c>
-      <c r="B95">
-        <v>0</v>
+      <c r="B95" s="2">
+        <v>42332714</v>
       </c>
       <c r="C95" s="2">
         <v>21208411</v>
       </c>
-      <c r="D95">
-        <v>0</v>
+      <c r="D95" s="2">
+        <v>41</v>
       </c>
       <c r="E95" s="2">
         <v>5285747</v>
       </c>
-      <c r="F95">
-        <v>0</v>
+      <c r="F95" s="2">
+        <v>108027831</v>
       </c>
       <c r="G95" s="2">
         <v>30409897</v>
       </c>
-      <c r="H95">
-        <v>0</v>
-      </c>
-      <c r="I95">
-        <v>0</v>
-      </c>
-      <c r="J95">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="H95" s="2">
+        <v>1857831</v>
+      </c>
+      <c r="I95" s="2">
+        <v>85</v>
+      </c>
+      <c r="J95" s="2">
+        <v>1750</v>
+      </c>
+      <c r="K95" s="2"/>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A96" s="1">
         <v>45838</v>
       </c>
-      <c r="B96">
-        <v>0</v>
+      <c r="B96" s="2">
+        <v>39571037</v>
       </c>
       <c r="C96" s="2">
         <v>21923522</v>
       </c>
-      <c r="D96">
-        <v>0</v>
+      <c r="D96" s="2">
+        <v>41</v>
       </c>
       <c r="E96" s="2">
         <v>5417822</v>
       </c>
-      <c r="F96">
-        <v>0</v>
+      <c r="F96" s="2">
+        <v>110397081</v>
       </c>
       <c r="G96" s="2">
         <v>30874034</v>
       </c>
-      <c r="H96">
-        <v>0</v>
-      </c>
-      <c r="I96">
-        <v>0</v>
-      </c>
-      <c r="J96">
-        <v>0</v>
-      </c>
+      <c r="H96" s="2">
+        <v>1859195</v>
+      </c>
+      <c r="I96" s="2">
+        <v>85</v>
+      </c>
+      <c r="J96" s="2">
+        <v>1750</v>
+      </c>
+      <c r="K96" s="2"/>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A97" s="1">
@@ -14006,7 +14020,7 @@
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A102" s="2">
+      <c r="A102" s="1">
         <v>46022</v>
       </c>
       <c r="B102" s="2">
@@ -14038,7 +14052,7 @@
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A103" s="2">
+      <c r="A103" s="1">
         <v>46053</v>
       </c>
       <c r="B103" s="2">
@@ -14070,7 +14084,7 @@
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A104" s="2">
+      <c r="A104" s="1">
         <v>46081</v>
       </c>
       <c r="B104" s="2">

</xml_diff>

<commit_message>
chore: re-generate migration scripts from corrected 데이터원본_2602.xlsx
GitHub main 브랜치의 최신 xlsx(25년11월~26년2월 toss 반영) 기준으로 재생성

https://claude.ai/code/session_013KN2ckCjgMsHNupTh13SeR
</commit_message>
<xml_diff>
--- a/데이터원본_2602.xlsx
+++ b/데이터원본_2602.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\내 드라이브\02_AREA\04_재무\04_연금전략 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{577F5B33-3C1A-416F-9B5E-1D6658105B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9ED602-8D9B-4DE5-9D8A-B99CA49FCA59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38350" yWindow="-16110" windowWidth="38620" windowHeight="15500" xr2:uid="{182F7363-D65B-489E-BF18-685EC1FD72DA}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{182F7363-D65B-489E-BF18-685EC1FD72DA}"/>
   </bookViews>
   <sheets>
     <sheet name="평가금액" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
-    <numFmt numFmtId="177" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -144,7 +144,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -13992,7 +13992,7 @@
         <v>45991</v>
       </c>
       <c r="B101" s="2">
-        <v>38678383</v>
+        <v>37947509</v>
       </c>
       <c r="C101" s="2">
         <v>27713408</v>
@@ -14004,13 +14004,13 @@
         <v>6310583</v>
       </c>
       <c r="F101" s="2">
-        <v>127264650</v>
+        <v>131001635</v>
       </c>
       <c r="G101" s="2">
         <v>35765466</v>
       </c>
       <c r="H101" s="2">
-        <v>1752252</v>
+        <v>1757136</v>
       </c>
       <c r="I101">
         <v>85</v>
@@ -14024,7 +14024,7 @@
         <v>46022</v>
       </c>
       <c r="B102" s="2">
-        <v>38678383</v>
+        <v>35483957</v>
       </c>
       <c r="C102" s="2">
         <v>28697525</v>
@@ -14036,13 +14036,13 @@
         <v>6363175</v>
       </c>
       <c r="F102" s="2">
-        <v>127264650</v>
+        <v>128856432</v>
       </c>
       <c r="G102" s="2">
         <v>35909101</v>
       </c>
       <c r="H102" s="2">
-        <v>1752252</v>
+        <v>1741194</v>
       </c>
       <c r="I102">
         <v>85</v>
@@ -14056,7 +14056,7 @@
         <v>46053</v>
       </c>
       <c r="B103" s="2">
-        <v>38678383</v>
+        <v>33104131</v>
       </c>
       <c r="C103" s="2">
         <v>30629637</v>
@@ -14068,13 +14068,13 @@
         <v>6427893</v>
       </c>
       <c r="F103" s="2">
-        <v>127264650</v>
+        <v>132876869</v>
       </c>
       <c r="G103" s="2">
         <v>36270455</v>
       </c>
       <c r="H103" s="2">
-        <v>1752252</v>
+        <v>1716779</v>
       </c>
       <c r="I103">
         <v>85</v>
@@ -14088,7 +14088,7 @@
         <v>46081</v>
       </c>
       <c r="B104" s="2">
-        <v>38678383</v>
+        <v>45047162</v>
       </c>
       <c r="C104" s="2">
         <v>31259926</v>
@@ -14100,13 +14100,13 @@
         <v>6396017</v>
       </c>
       <c r="F104" s="2">
-        <v>127264650</v>
+        <v>137359977</v>
       </c>
       <c r="G104" s="2">
         <v>35702242</v>
       </c>
       <c r="H104" s="2">
-        <v>1752252</v>
+        <v>1681273</v>
       </c>
       <c r="I104">
         <v>85</v>

</xml_diff>